<commit_message>
revisi testing model dengan data baru 2026
</commit_message>
<xml_diff>
--- a/output/rekap_produk.xlsx
+++ b/output/rekap_produk.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B262"/>
+  <dimension ref="A1:B177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,17 +435,17 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>232</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>daily ceramois hydra gel</t>
+          <t>radian brightening ultimate</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>223</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4">
@@ -455,27 +455,27 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>220</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>hb dosting 75 gram</t>
+          <t>paket brightening</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>197</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>paket brightening</t>
+          <t>daily ceramois hydra gel</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>173</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7">
@@ -485,717 +485,717 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>165</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>dna salmon extra marine collagen and hyaluronic acid 30 ml</t>
+          <t>paket radiant brightening ultimate</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>158</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>radian brightening ultimate</t>
+          <t>hb dosting 75 gram</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>148</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>serum brightening glowing</t>
+          <t>sunscreen glowing new</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>145</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>sunscreen glowing new</t>
+          <t>dna salmon extra marine collagen and hyaluronic acid 30 ml</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>141</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>paket custom</t>
+          <t>sunscreen natural glow for normal skin new</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>128</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>paket acne 1</t>
+          <t>serum for acne skin new</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>122</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sunscreen natural glow for normal skin new</t>
+          <t>serum brightening glowing</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>115</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sunscreen for oily &amp; acne</t>
+          <t>night cream acne brightening</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>105</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>luminous brightening vitamin c plus collagen serum</t>
+          <t>sunscreen yellow glow new</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>100</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>brightening 3</t>
+          <t>paket acne 1</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>99</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>milk cleanser 110 ml</t>
+          <t>hb night yellow plus licorice</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>paket hb lotion yellow+licorice</t>
+          <t>hb night brightening</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>85</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>paket radiant brightening ultimate</t>
+          <t>paket radian brightening ultimate</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>83</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>toner honey premium 110 ml new</t>
+          <t>paket acne brightening</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>82</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>sunscreen yellow glow new</t>
+          <t>milk cleanser 110 ml</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>81</v>
+        <v>43</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>toner lime premium 110 ml new</t>
+          <t>paket custom</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>79</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>paket radian brightening ultimate</t>
+          <t>bb chusion flawless</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>79</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>acne cream 1 new</t>
+          <t>toner honey premium 110 ml new</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>74</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>radian acne brightening new</t>
+          <t>paket hb dosting</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>72</v>
+        <v>41</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>night cream acne brightening</t>
+          <t>radian glow booster (rgb)</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>70</v>
+        <v>36</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>serum for acne skin new</t>
+          <t>facial wash for normal skin 110 ml new</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>70</v>
+        <v>34</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>serum for acne skin</t>
+          <t>toner lime premium 110 ml new</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>69</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>paket ceramois acne</t>
+          <t>luminous brightening vitamin c plus collagen serum</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>66</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>tenteng motif</t>
+          <t>acne cream 2 new</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>65</v>
+        <v>33</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>sunscreen natural glow for normal skin</t>
+          <t>acne cream 1 new</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>64</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>paket acne brightening</t>
+          <t>brightening cream 1 with licorice plus astaxanthin</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>64</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>radian brightening</t>
+          <t>glowtech spicule rejuvenation</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>63</v>
+        <v>31</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>paket radian acne brightening</t>
+          <t>lips care new</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>62</v>
+        <v>28</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>night cream acne</t>
+          <t>paket acne</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>62</v>
+        <v>27</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>acne cream 2 new</t>
+          <t>paket radiant glow booster</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>amour matte lip cream</t>
+          <t>hydrating essence toner 10x amino acid</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>cermin croco drw</t>
+          <t>sabun kojic milk</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>facial wash for normal skin 110 ml new</t>
+          <t>bb chusion ivory</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>toner lime 110 ml</t>
+          <t>drw goats milk body lotion</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>56</v>
+        <v>24</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>paket acne 2</t>
+          <t>night cream acne</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>55</v>
+        <v>24</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>paket hb dosting</t>
+          <t>brightening cream 2 alpha arbutin + shea butter</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>54</v>
+        <v>24</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>paket radian brightening</t>
+          <t>day cream pink new</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>53</v>
+        <v>22</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>sunscreen glowing</t>
+          <t>paket brightening 1</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>52</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>brightening cream 2 alpha arbutin + shea butter</t>
+          <t>glu glow drink rasa blackcurrant</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>51</v>
+        <v>21</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>lips care new</t>
+          <t>brightening 3</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>50</v>
+        <v>19</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>brightening cream 1 with licorice plus astaxanthin</t>
+          <t>facial wash pink brightening 110 ml new</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>49</v>
+        <v>19</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>paket ceramois glowing</t>
+          <t>paket hemat acne 2</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>toner brightening</t>
+          <t>bedak tabur natural</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>paket brightening 1</t>
+          <t>paket hemat brightening 1</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>brightening cream with licorice plus astaxanthin</t>
+          <t>paket hemat acne 1</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>48</v>
+        <v>17</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>hb night rejuvenation</t>
+          <t>day acne 1 new</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>radian acne brigh</t>
+          <t>amour matte lip cream</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>46</v>
+        <v>17</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>toner honey 110 ml</t>
+          <t>paket acne 2</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>44</v>
+        <v>16</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>hydrating essence toner 10x amino acid</t>
+          <t>flimeberry rasa strawberry</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>44</v>
+        <v>15</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>hb night brightening</t>
+          <t>paket brightening 3</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>43</v>
+        <v>15</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>paket acne 3</t>
+          <t>serum aha bha new</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>43</v>
+        <v>14</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>hb night yellow plus licorice</t>
+          <t>body lotion tone up 100 ml</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>42</v>
+        <v>14</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>paperbag</t>
+          <t>lipgloss gold new</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>42</v>
+        <v>14</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>paket hemat acne 1</t>
+          <t>paket brightening 2</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>41</v>
+        <v>13</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>clutch mini croco</t>
+          <t>paket ceramois acne</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>40</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>paket radian acne</t>
+          <t>facial wash oily acne 63 ml new</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>40</v>
+        <v>13</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>brightening cream alpha arbutin + shea butter</t>
+          <t>cnr + calming and rejuvenation cream</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>40</v>
+        <v>13</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>paket brightening 3</t>
+          <t>paket ceramois glowing</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>39</v>
+        <v>13</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>facial wash pink brightening 110 ml new</t>
+          <t>acne cream 3 new</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>38</v>
+        <v>12</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>day cream pink new</t>
+          <t>toner lime premium 63 ml new</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>38</v>
+        <v>12</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>bb chusion flawless</t>
+          <t>paket hemat brightening 2</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>radian glow</t>
+          <t>bloome micellar water</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>day acne 1 new</t>
+          <t>kapas kecantikan modis 50 gr</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>35</v>
+        <v>11</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>hb day foundation</t>
+          <t>radiant acne repair</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>drw goats milk body lotion</t>
+          <t>toner honey premium 63 ml new</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>sabun kojic milk</t>
+          <t>facial wash tea tree oil 110 ml new</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>snail anti aging</t>
+          <t>serum brightening with vit c and e new</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>acne cream 3 new</t>
+          <t>paket glow maksimal</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>paket brightening 2</t>
+          <t>snail anti aging new</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>day cream white new</t>
+          <t>paket hemat rbu</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>paket acne</t>
+          <t>drw slimming capsule</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>31</v>
+        <v>9</v>
       </c>
     </row>
     <row r="79">
@@ -1205,1836 +1205,986 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>facial wash pink bright 110 ml</t>
+          <t>facial wash for normal skin 63 ml new</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>29</v>
+        <v>9</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>bedak tabur natural</t>
+          <t>paket hemat brightening 3</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>snail anti aging new</t>
+          <t>day cream white new</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>acne 1</t>
+          <t>milk cleanser 63 ml</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>facial wash oily acne 63 ml new</t>
+          <t>sabun bamboo charcoal</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>milk cleanser 63 ml</t>
+          <t>micellar water 100 ml</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>paperbag besar</t>
+          <t>paket bye flek</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>paket hemat brightening 2</t>
+          <t>paket flek luntur</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>sunscreen yellow glow</t>
+          <t>bedak tabur beige</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>drw slimming capsule</t>
+          <t>lipgloss pink new</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>paket radian glow</t>
+          <t>paket acne 3</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>serum aha bha new</t>
+          <t>kapsul gemuk</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>paket hemat acne 3</t>
+          <t>bedak tabur ivory</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>radian acne</t>
+          <t>anti aging eye gel</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>paket hemat brightening 3</t>
+          <t>paket radiant acne repair</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>bedak padat (beige)</t>
+          <t>toner chamomile 110 ml new</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>toner chamomile 110 ml new</t>
+          <t>facial wash white formen</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>serum retinol</t>
+          <t>exfoliating complex toner aha bha pha</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>toner lime premium 63 ml new</t>
+          <t>kapas kecantikan modis 85 gr</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>toner honey premium 63 ml new</t>
+          <t>new beauty dna salmon spray</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>susu d'etawa plus collagen rasa strawberry</t>
+          <t>day acne 2 new</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>facial wash for normal skin 110 ml</t>
+          <t>toner lime 110 ml</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>tenteng polos</t>
+          <t>snail anti aging</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>paket hb rejuvenation</t>
+          <t>facial wash pink brightening 63 ml new</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>paket hemat rad acne bright</t>
+          <t>toner chamomile 63 ml new</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>paket hemat acne 2</t>
+          <t>paket hemat acne 3</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>paket hemat brightening 1</t>
+          <t>kapas kecantikan modis 35 gr</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>radian brightening new</t>
+          <t>3 in 1 exfoliating gel 100 ml</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>sabun bamboo charcoal</t>
+          <t>facemist 100 ml</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>day acne 1</t>
+          <t>deo herba strong</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>bedak tabur ivory</t>
+          <t>sunscreen pinky glow new</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>3 in 1 exfoliating gel 100 ml</t>
+          <t>peel off mask for oily and acne skin 60 ml</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>facial wash tea tree oil 110 ml new</t>
+          <t>paket goats milk series</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>acne 2</t>
+          <t>paket bye jerawat</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>peel off mask for oily and acne skin 60 ml</t>
+          <t>sunscreen normal skin for men</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>sunscreen pinky glow</t>
+          <t>serum retinol</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>facial wash for normal skin 63 ml new</t>
+          <t>dompet premium</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>facial wash white formen</t>
+          <t>paket serum custom</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>body lotion tone up 100 ml</t>
+          <t>paket rgb + dna salmon</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>paket goats milk series</t>
+          <t>paket anti kusam</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>clutch mini butterfly</t>
+          <t>exfoliating derma essence aha bha pha</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>day cream white</t>
+          <t>drw goats milk body wash</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>serum brightening with vit c and e new</t>
+          <t>paket snail cream</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>paket hemat rad glow</t>
+          <t>snail cream anti aging new</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>brightening 1</t>
+          <t>fragile</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>day acne 2 new</t>
+          <t>hair serum premium</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>acne 3</t>
+          <t>cnr plus calming and rejuvenation cream</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>facemist 100 ml</t>
+          <t>kapas 80gr</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>bedak padat (natural)</t>
+          <t>lulur brightening premium</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>dompet premium</t>
+          <t>lipgloss beauty pink</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>day cream pink</t>
+          <t>susu d'etawa plus collagen rasa strawberry</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>beauty dna salmon spray</t>
+          <t>paket kulit tenang</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>paket hemat rad bright</t>
+          <t>d etawa susu etawa plus collagen rasa brown sugar</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>radian glow new</t>
+          <t>exfoliating gel</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>hb day premium</t>
+          <t>treatment</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>sunscreen normal skin for men</t>
+          <t>facial wash pink bright 63 ml</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>bb chusion ivory</t>
+          <t>miceller water 63 ml</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>paket hemat rad acne</t>
+          <t>facial wash oily acne 63 ml</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>bedak padat (pink)</t>
+          <t>shampo aleovera+ conditioner 200 ml</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>anti aging eye gel</t>
+          <t>moisturizel gel</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>kapas kecantikan modis 50 gr</t>
+          <t>lipgloss beauty gold</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>underarm cream</t>
+          <t>drw goats milk body scrub</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>drw goats milk body wash</t>
+          <t>stretchmark cream</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>paket brightening cream</t>
+          <t>sunscreen oily acne for men</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>micellar water 100 ml</t>
+          <t>facial wash pink bright 110 ml</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>radian glow booster (rgb)</t>
+          <t>breast cream</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>facial wash oily acne 63 ml</t>
+          <t>brightening peel off mask with charcoal 60 ml</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>d etawa susu etawa plus collagen rasa brown sugar</t>
+          <t>sunscreen natural glow for normal skin</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>night cream for men</t>
+          <t>kapas modis 80g</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>ongkir spx</t>
+          <t>body firming cream</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>lipgloss beauty pink</t>
+          <t>drw glutation</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>brightening 2</t>
+          <t>paket soft glow + dna salmon</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>brightening peel off mask with charcoal 60 ml</t>
+          <t>paket acne series + serum</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>sunscreen oily acne for men</t>
+          <t>paket hemat ncf</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>serum aha bha</t>
+          <t>chibao</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>glowtech spicule rejuvenation</t>
+          <t>chibao grey</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>moisturizel gel</t>
+          <t>paket awet muda</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>facial wash tea tree oil 63 ml new</t>
+          <t>cek kulit skin analyzer</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>sabun kojic sulfur</t>
+          <t>paket cerah body &amp; lips</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>deo herba strong</t>
+          <t>serum aha bha</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>drw glutation</t>
+          <t>radian acne brigh</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>lipgloss gold new</t>
+          <t>toner brightening</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>paket hemat rbu</t>
+          <t>masker green tea</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>toner chamomile 110 ml</t>
+          <t>micellar water for men 100 ml</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>cermin bulat</t>
+          <t>kapas kecantikan 80 gr</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>facial wash oily acne 110 ml</t>
+          <t>facial wash for normal skin 63 ml</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>brosur kecil (10 lembar)</t>
+          <t>sunscreen glowing</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>radian acne new</t>
+          <t>day acne 3 new</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>bedak padat (kotak)</t>
+          <t>kapas 80g</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>dermabright</t>
+          <t>modis 80g</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>toner honey 63 ml</t>
+          <t>obat jerawat (poc)</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>treatment</t>
+          <t>bedak padat (pink)</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>day acne 3 new</t>
+          <t>paket hb lotion yellow+licorice</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>facial wash tto 110 ml</t>
+          <t>facial wash tea tree oil 63 ml new</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>serum scar</t>
+          <t>brightening cream with licorice plus astaxanthin</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>bedak tabur beige</t>
+          <t>afen</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>lulur brightening premium</t>
+          <t>sabun kojic sulfur</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>paket snail cream</t>
+          <t>shampo anti dandruf</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>paket serum custom</t>
-        </is>
-      </c>
-      <c r="B178" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>paket hemat ncf</t>
-        </is>
-      </c>
-      <c r="B179" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>paket hemat nacf</t>
-        </is>
-      </c>
-      <c r="B180" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>ongkir jnt vip</t>
-        </is>
-      </c>
-      <c r="B181" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>sunscreen pinky glow new</t>
-        </is>
-      </c>
-      <c r="B182" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>lipgloss pink new</t>
-        </is>
-      </c>
-      <c r="B183" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>toner chamomile 63 ml new</t>
-        </is>
-      </c>
-      <c r="B184" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>body firming cream</t>
-        </is>
-      </c>
-      <c r="B185" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>breast cream</t>
-        </is>
-      </c>
-      <c r="B186" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>stretchmark cream</t>
-        </is>
-      </c>
-      <c r="B187" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>neck cream brightening</t>
-        </is>
-      </c>
-      <c r="B188" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>day acne 3</t>
-        </is>
-      </c>
-      <c r="B189" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>exfoliating derma essence aha bha pha</t>
-        </is>
-      </c>
-      <c r="B190" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>day acne 2</t>
-        </is>
-      </c>
-      <c r="B191" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>kapas kecantikan modis 35 gr</t>
-        </is>
-      </c>
-      <c r="B192" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>paket hemat custom</t>
-        </is>
-      </c>
-      <c r="B193" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>masker green tea</t>
-        </is>
-      </c>
-      <c r="B194" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>hair tonic normal</t>
-        </is>
-      </c>
-      <c r="B195" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>exfoliating gel</t>
-        </is>
-      </c>
-      <c r="B196" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>facial wash tto 63 ml</t>
-        </is>
-      </c>
-      <c r="B197" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>brosur a4 drw</t>
-        </is>
-      </c>
-      <c r="B198" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>kapsul gemuk</t>
-        </is>
-      </c>
-      <c r="B199" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>d'etawa susu etawa plus collagen rasa original stevia</t>
-        </is>
-      </c>
-      <c r="B200" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>toner lime 63 ml</t>
-        </is>
-      </c>
-      <c r="B201" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>cek kulit skin analyzer</t>
-        </is>
-      </c>
-      <c r="B202" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>snail cream anti aging new</t>
-        </is>
-      </c>
-      <c r="B203" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>spesialis flek (premium)</t>
-        </is>
-      </c>
-      <c r="B204" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>paket acne bright for men</t>
-        </is>
-      </c>
-      <c r="B205" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>facial wash pink brightening 63 ml new</t>
-        </is>
-      </c>
-      <c r="B206" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>paket acne for men</t>
-        </is>
-      </c>
-      <c r="B207" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>paket alternatif glow and brightening 2</t>
-        </is>
-      </c>
-      <c r="B208" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>lakban fragile</t>
-        </is>
-      </c>
-      <c r="B209" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>ongkir</t>
-        </is>
-      </c>
-      <c r="B210" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>deo herba coolbright</t>
-        </is>
-      </c>
-      <c r="B211" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>lipgloss beauty gold</t>
-        </is>
-      </c>
-      <c r="B212" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>paket bright glow 3</t>
-        </is>
-      </c>
-      <c r="B213" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>paket glow for men</t>
-        </is>
-      </c>
-      <c r="B214" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>paket shampoo</t>
-        </is>
-      </c>
-      <c r="B215" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>new beauty dna salmon spray</t>
-        </is>
-      </c>
-      <c r="B216" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>micellar water for men 100 ml</t>
-        </is>
-      </c>
-      <c r="B217" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>hair serum premium</t>
-        </is>
-      </c>
-      <c r="B218" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>masker tea tree oil</t>
-        </is>
-      </c>
-      <c r="B219" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>paket hemat rg/rb+milkcleanser</t>
-        </is>
-      </c>
-      <c r="B220" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>shampo aleovera+ conditioner 200 ml</t>
-        </is>
-      </c>
-      <c r="B221" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>ongkir jnt cod vip</t>
-        </is>
-      </c>
-      <c r="B222" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>ongkir cod vip</t>
-        </is>
-      </c>
-      <c r="B223" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="inlineStr">
-        <is>
-          <t>lakban bening</t>
-        </is>
-      </c>
-      <c r="B224" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="inlineStr">
-        <is>
-          <t>exfoliating complex toner aha bha pha</t>
-        </is>
-      </c>
-      <c r="B225" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="inlineStr">
-        <is>
-          <t>spesialis bebas flek,keriput &amp; cerah ( glow up)</t>
-        </is>
-      </c>
-      <c r="B226" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>paket flek ringan</t>
-        </is>
-      </c>
-      <c r="B227" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>paket flek berat</t>
-        </is>
-      </c>
-      <c r="B228" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="inlineStr">
-        <is>
-          <t>paket alternatif glow and brightening</t>
-        </is>
-      </c>
-      <c r="B229" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="inlineStr">
-        <is>
-          <t>facial wash for normal skin 63 ml</t>
-        </is>
-      </c>
-      <c r="B230" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" t="inlineStr">
-        <is>
-          <t>paket hemat rg/rb miceller</t>
-        </is>
-      </c>
-      <c r="B231" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" t="inlineStr">
-        <is>
-          <t>paket oily 4 acne bha 60 ml</t>
-        </is>
-      </c>
-      <c r="B232" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" t="inlineStr">
-        <is>
-          <t>paket hemat ra/rab miceller</t>
-        </is>
-      </c>
-      <c r="B233" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" t="inlineStr">
-        <is>
-          <t>lips cream matte</t>
-        </is>
-      </c>
-      <c r="B234" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" t="inlineStr">
-        <is>
-          <t>paket micellar water for men</t>
-        </is>
-      </c>
-      <c r="B235" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" t="inlineStr">
-        <is>
-          <t>facial wash normal skin 110 ml</t>
-        </is>
-      </c>
-      <c r="B236" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" t="inlineStr">
-        <is>
-          <t>bb cushion ivory</t>
-        </is>
-      </c>
-      <c r="B237" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" t="inlineStr">
-        <is>
-          <t>clutch tali premium</t>
-        </is>
-      </c>
-      <c r="B238" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" t="inlineStr">
-        <is>
-          <t>ongkir jnt apk 40%</t>
-        </is>
-      </c>
-      <c r="B239" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" t="inlineStr">
-        <is>
-          <t>ongkir jnt vip cod</t>
-        </is>
-      </c>
-      <c r="B240" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" t="inlineStr">
-        <is>
-          <t>toner chamomile 63 ml</t>
-        </is>
-      </c>
-      <c r="B241" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" t="inlineStr">
-        <is>
-          <t>paket dermabright</t>
-        </is>
-      </c>
-      <c r="B242" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" t="inlineStr">
-        <is>
-          <t>paket brightening for men</t>
-        </is>
-      </c>
-      <c r="B243" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" t="inlineStr">
-        <is>
-          <t>lipskrim</t>
-        </is>
-      </c>
-      <c r="B244" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" t="inlineStr">
-        <is>
-          <t>treatment ketiak 3x ipl</t>
-        </is>
-      </c>
-      <c r="B245" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" t="inlineStr">
-        <is>
-          <t>radian glow brightening (rgb)</t>
-        </is>
-      </c>
-      <c r="B246" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" t="inlineStr">
-        <is>
-          <t>pdt treatment</t>
-        </is>
-      </c>
-      <c r="B247" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" t="inlineStr">
-        <is>
-          <t>miceller water 63 ml</t>
-        </is>
-      </c>
-      <c r="B248" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" t="inlineStr">
-        <is>
-          <t>paket hemat nac</t>
-        </is>
-      </c>
-      <c r="B249" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" t="inlineStr">
-        <is>
-          <t>drw goats milk body scrub</t>
-        </is>
-      </c>
-      <c r="B250" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" t="inlineStr">
-        <is>
-          <t>paket cream farmasi</t>
-        </is>
-      </c>
-      <c r="B251" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="inlineStr">
-        <is>
-          <t>paket cream racik</t>
-        </is>
-      </c>
-      <c r="B252" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="inlineStr">
-        <is>
-          <t>jnt</t>
-        </is>
-      </c>
-      <c r="B253" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" t="inlineStr">
-        <is>
-          <t>spesialis bebas garis halus kencang dan tirus (premium)</t>
-        </is>
-      </c>
-      <c r="B254" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" t="inlineStr">
-        <is>
-          <t>tambahan treatment</t>
-        </is>
-      </c>
-      <c r="B255" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" t="inlineStr">
-        <is>
-          <t>spesialis flek (spekta)</t>
-        </is>
-      </c>
-      <c r="B256" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" t="inlineStr">
-        <is>
-          <t>rf slimming seluruh wajah</t>
-        </is>
-      </c>
-      <c r="B257" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" t="inlineStr">
-        <is>
-          <t>masker peel off pink</t>
-        </is>
-      </c>
-      <c r="B258" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="inlineStr">
-        <is>
-          <t>facial white</t>
-        </is>
-      </c>
-      <c r="B259" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="inlineStr">
-        <is>
-          <t>hydra peel</t>
-        </is>
-      </c>
-      <c r="B260" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" t="inlineStr">
-        <is>
-          <t>detok ketiak / underarm</t>
-        </is>
-      </c>
-      <c r="B261" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="inlineStr">
-        <is>
-          <t>detox wajah</t>
-        </is>
-      </c>
-      <c r="B262" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>